<commit_message>
chore: consolidate experiment workspace and results
</commit_message>
<xml_diff>
--- a/ZAC_zzx/results/fourway/四方法_对齐TableI.xlsx
+++ b/ZAC_zzx/results/fourway/四方法_对齐TableI.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W27"/>
+  <dimension ref="A1:W28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1964,38 +1964,57 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>geomean Steps/ZAC</t>
+          <t>平均保真度(N=18 N=2)</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>0.6038</v>
       </c>
       <c r="C26" t="n">
-        <v>0.858</v>
+        <v>0.5485</v>
       </c>
       <c r="D26" t="n">
-        <v>0.92</v>
+        <v>0.6195000000000001</v>
       </c>
       <c r="E26" t="n">
-        <v>0.914</v>
+        <v>0.6193</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>geomean Rearr/ZAC</t>
+          <t>geomean Steps/ZAC</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>1</v>
       </c>
       <c r="C27" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.914</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>geomean Rearr/ZAC</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
         <v>0.859</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D28" t="n">
         <v>0.99</v>
       </c>
-      <c r="E27" t="n">
+      <c r="E28" t="n">
         <v>0.985</v>
       </c>
     </row>
@@ -2013,7 +2032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U163"/>
+  <dimension ref="A1:U164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2184,10 +2203,10 @@
         <v>16.38</v>
       </c>
       <c r="J3" t="n">
-        <v>27.576</v>
+        <v>28.465</v>
       </c>
       <c r="K3" t="n">
-        <v>0.032</v>
+        <v>0.042</v>
       </c>
       <c r="L3" t="n">
         <v>152</v>
@@ -2251,10 +2270,10 @@
         <v>2.97</v>
       </c>
       <c r="J4" t="n">
-        <v>5.427</v>
+        <v>5.929</v>
       </c>
       <c r="K4" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
       <c r="L4" t="n">
         <v>32</v>
@@ -2318,10 +2337,10 @@
         <v>17.03</v>
       </c>
       <c r="J5" t="n">
-        <v>30.301</v>
+        <v>31.243</v>
       </c>
       <c r="K5" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="L5" t="n">
         <v>179</v>
@@ -2385,10 +2404,10 @@
         <v>11.49</v>
       </c>
       <c r="J6" t="n">
-        <v>20.618</v>
+        <v>21.047</v>
       </c>
       <c r="K6" t="n">
-        <v>0.015</v>
+        <v>0.017</v>
       </c>
       <c r="L6" t="n">
         <v>121</v>
@@ -2452,7 +2471,7 @@
         <v>2.39</v>
       </c>
       <c r="J7" t="n">
-        <v>4.994</v>
+        <v>5.303</v>
       </c>
       <c r="K7" t="n">
         <v>0.005</v>
@@ -2519,7 +2538,7 @@
         <v>2.17</v>
       </c>
       <c r="J8" t="n">
-        <v>4.515</v>
+        <v>4.909</v>
       </c>
       <c r="K8" t="n">
         <v>0.004</v>
@@ -2586,10 +2605,10 @@
         <v>1.59</v>
       </c>
       <c r="J9" t="n">
-        <v>2.63</v>
+        <v>2.768</v>
       </c>
       <c r="K9" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="L9" t="n">
         <v>16</v>
@@ -2653,7 +2672,7 @@
         <v>18.24</v>
       </c>
       <c r="J10" t="n">
-        <v>32.705</v>
+        <v>34.303</v>
       </c>
       <c r="K10" t="n">
         <v>0.026</v>
@@ -2720,10 +2739,10 @@
         <v>18.03</v>
       </c>
       <c r="J11" t="n">
-        <v>32.345</v>
+        <v>33.848</v>
       </c>
       <c r="K11" t="n">
-        <v>0.023</v>
+        <v>0.03</v>
       </c>
       <c r="L11" t="n">
         <v>189</v>
@@ -2787,10 +2806,10 @@
         <v>14.89</v>
       </c>
       <c r="J12" t="n">
-        <v>26.248</v>
+        <v>27.148</v>
       </c>
       <c r="K12" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="L12" t="n">
         <v>156</v>
@@ -2854,10 +2873,10 @@
         <v>19.28</v>
       </c>
       <c r="J13" t="n">
-        <v>30.64</v>
+        <v>31.916</v>
       </c>
       <c r="K13" t="n">
-        <v>0.023</v>
+        <v>0.027</v>
       </c>
       <c r="L13" t="n">
         <v>181</v>
@@ -2921,10 +2940,10 @@
         <v>5.15</v>
       </c>
       <c r="J14" t="n">
-        <v>9.635999999999999</v>
+        <v>10.067</v>
       </c>
       <c r="K14" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="L14" t="n">
         <v>55</v>
@@ -2988,10 +3007,10 @@
         <v>8.85</v>
       </c>
       <c r="J15" t="n">
-        <v>15.071</v>
+        <v>15.665</v>
       </c>
       <c r="K15" t="n">
-        <v>0.011</v>
+        <v>0.014</v>
       </c>
       <c r="L15" t="n">
         <v>86</v>
@@ -3055,10 +3074,10 @@
         <v>8.85</v>
       </c>
       <c r="J16" t="n">
-        <v>15</v>
+        <v>15.74</v>
       </c>
       <c r="K16" t="n">
-        <v>0.011</v>
+        <v>0.014</v>
       </c>
       <c r="L16" t="n">
         <v>86</v>
@@ -3122,7 +3141,7 @@
         <v>5.37</v>
       </c>
       <c r="J17" t="n">
-        <v>9.483000000000001</v>
+        <v>9.436999999999999</v>
       </c>
       <c r="K17" t="n">
         <v>0.011</v>
@@ -3189,10 +3208,10 @@
         <v>19.37</v>
       </c>
       <c r="J18" t="n">
-        <v>32.757</v>
+        <v>33.931</v>
       </c>
       <c r="K18" t="n">
-        <v>0.027</v>
+        <v>0.026</v>
       </c>
       <c r="L18" t="n">
         <v>193</v>
@@ -3256,10 +3275,10 @@
         <v>29.69</v>
       </c>
       <c r="J19" t="n">
-        <v>54.335</v>
+        <v>55.747</v>
       </c>
       <c r="K19" t="n">
-        <v>0.032</v>
+        <v>0.039</v>
       </c>
       <c r="L19" t="n">
         <v>316</v>
@@ -3323,10 +3342,10 @@
         <v>18.35</v>
       </c>
       <c r="J20" t="n">
-        <v>33.009</v>
+        <v>34.528</v>
       </c>
       <c r="K20" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="L20" t="n">
         <v>192</v>
@@ -3390,10 +3409,10 @@
         <v>17.65</v>
       </c>
       <c r="J21" t="n">
-        <v>31.498</v>
+        <v>33.131</v>
       </c>
       <c r="K21" t="n">
-        <v>0.019</v>
+        <v>0.027</v>
       </c>
       <c r="L21" t="n">
         <v>184</v>
@@ -3457,10 +3476,10 @@
         <v>14.02</v>
       </c>
       <c r="J22" t="n">
-        <v>24.094</v>
+        <v>28.426</v>
       </c>
       <c r="K22" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="L22" t="n">
         <v>145</v>
@@ -3524,10 +3543,10 @@
         <v>21.8</v>
       </c>
       <c r="J23" t="n">
-        <v>36.674</v>
+        <v>38.97</v>
       </c>
       <c r="K23" t="n">
-        <v>0.025</v>
+        <v>0.029</v>
       </c>
       <c r="L23" t="n">
         <v>221</v>
@@ -3591,10 +3610,10 @@
         <v>6.48</v>
       </c>
       <c r="J24" t="n">
-        <v>11.701</v>
+        <v>12.111</v>
       </c>
       <c r="K24" t="n">
-        <v>0.011</v>
+        <v>0.014</v>
       </c>
       <c r="L24" t="n">
         <v>68</v>
@@ -3658,10 +3677,10 @@
         <v>7.31</v>
       </c>
       <c r="J25" t="n">
-        <v>14.256</v>
+        <v>14.573</v>
       </c>
       <c r="K25" t="n">
-        <v>0.011</v>
+        <v>0.014</v>
       </c>
       <c r="L25" t="n">
         <v>77</v>
@@ -3725,10 +3744,10 @@
         <v>9.970000000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>17.333</v>
+        <v>18.323</v>
       </c>
       <c r="K26" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="L26" t="n">
         <v>105</v>
@@ -3792,10 +3811,10 @@
         <v>6.04</v>
       </c>
       <c r="J27" t="n">
-        <v>10.436</v>
+        <v>10.872</v>
       </c>
       <c r="K27" t="n">
-        <v>0.006</v>
+        <v>0.008</v>
       </c>
       <c r="L27" t="n">
         <v>60</v>
@@ -3859,10 +3878,10 @@
         <v>5.29</v>
       </c>
       <c r="J28" t="n">
-        <v>10.12</v>
+        <v>10.828</v>
       </c>
       <c r="K28" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="L28" t="n">
         <v>56</v>
@@ -3926,10 +3945,10 @@
         <v>3.1</v>
       </c>
       <c r="J29" t="n">
-        <v>5.307</v>
+        <v>5.943</v>
       </c>
       <c r="K29" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="L29" t="n">
         <v>32</v>
@@ -3993,10 +4012,10 @@
         <v>2.13</v>
       </c>
       <c r="J30" t="n">
-        <v>3.53</v>
+        <v>3.663</v>
       </c>
       <c r="K30" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
       <c r="L30" t="n">
         <v>17</v>
@@ -4060,10 +4079,10 @@
         <v>2.01</v>
       </c>
       <c r="J31" t="n">
-        <v>3.844</v>
+        <v>3.882</v>
       </c>
       <c r="K31" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="L31" t="n">
         <v>19</v>
@@ -4127,7 +4146,7 @@
         <v>5.76</v>
       </c>
       <c r="J32" t="n">
-        <v>9.984</v>
+        <v>10.366</v>
       </c>
       <c r="K32" t="n">
         <v>0.011</v>
@@ -4194,10 +4213,10 @@
         <v>3.11</v>
       </c>
       <c r="J33" t="n">
-        <v>5.569</v>
+        <v>5.661</v>
       </c>
       <c r="K33" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="L33" t="n">
         <v>31</v>
@@ -4261,10 +4280,10 @@
         <v>12.18</v>
       </c>
       <c r="J34" t="n">
-        <v>21.824</v>
+        <v>22.513</v>
       </c>
       <c r="K34" t="n">
-        <v>0.018</v>
+        <v>0.019</v>
       </c>
       <c r="L34" t="n">
         <v>127</v>
@@ -4328,10 +4347,10 @@
         <v>15.12</v>
       </c>
       <c r="J35" t="n">
-        <v>20.738</v>
+        <v>21.431</v>
       </c>
       <c r="K35" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="L35" t="n">
         <v>126</v>
@@ -4403,10 +4422,10 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>4495.008</v>
+        <v>4561.676</v>
       </c>
       <c r="K36" t="n">
-        <v>3.621</v>
+        <v>3.276</v>
       </c>
       <c r="L36" t="n">
         <v>26800</v>
@@ -4486,10 +4505,10 @@
         <v>34.77</v>
       </c>
       <c r="J37" t="n">
-        <v>60.601</v>
+        <v>62.224</v>
       </c>
       <c r="K37" t="n">
-        <v>0.06</v>
+        <v>0.051</v>
       </c>
       <c r="L37" t="n">
         <v>364</v>
@@ -4553,10 +4572,10 @@
         <v>256.72</v>
       </c>
       <c r="J38" t="n">
-        <v>429.958</v>
+        <v>442.47</v>
       </c>
       <c r="K38" t="n">
-        <v>0.339</v>
+        <v>0.35</v>
       </c>
       <c r="L38" t="n">
         <v>2612</v>
@@ -4620,10 +4639,10 @@
         <v>12.8</v>
       </c>
       <c r="J39" t="n">
-        <v>21.261</v>
+        <v>22.113</v>
       </c>
       <c r="K39" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="L39" t="n">
         <v>127</v>
@@ -4687,10 +4706,10 @@
         <v>7.01</v>
       </c>
       <c r="J40" t="n">
-        <v>20.598</v>
+        <v>21.72</v>
       </c>
       <c r="K40" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="L40" t="n">
         <v>70</v>
@@ -4754,7 +4773,7 @@
         <v>6.93</v>
       </c>
       <c r="J41" t="n">
-        <v>11.862</v>
+        <v>12.089</v>
       </c>
       <c r="K41" t="n">
         <v>0.012</v>
@@ -4821,7 +4840,7 @@
         <v>3.06</v>
       </c>
       <c r="J42" t="n">
-        <v>5.11</v>
+        <v>5.286</v>
       </c>
       <c r="K42" t="n">
         <v>0.005</v>
@@ -4888,10 +4907,10 @@
         <v>3.07</v>
       </c>
       <c r="J43" t="n">
-        <v>5.509</v>
+        <v>5.568</v>
       </c>
       <c r="K43" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="L43" t="n">
         <v>30</v>
@@ -4955,10 +4974,10 @@
         <v>3.06</v>
       </c>
       <c r="J44" t="n">
-        <v>5.084</v>
+        <v>5.457</v>
       </c>
       <c r="K44" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="L44" t="n">
         <v>30</v>
@@ -5022,10 +5041,10 @@
         <v>37.48</v>
       </c>
       <c r="J45" t="n">
-        <v>66.754</v>
+        <v>68.342</v>
       </c>
       <c r="K45" t="n">
-        <v>0.044</v>
+        <v>0.047</v>
       </c>
       <c r="L45" t="n">
         <v>393</v>
@@ -5089,10 +5108,10 @@
         <v>32.9</v>
       </c>
       <c r="J46" t="n">
-        <v>58.492</v>
+        <v>60.779</v>
       </c>
       <c r="K46" t="n">
-        <v>0.041</v>
+        <v>0.045</v>
       </c>
       <c r="L46" t="n">
         <v>347</v>
@@ -5156,10 +5175,10 @@
         <v>12.89</v>
       </c>
       <c r="J47" t="n">
-        <v>22.203</v>
+        <v>22.444</v>
       </c>
       <c r="K47" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
       <c r="L47" t="n">
         <v>132</v>
@@ -5223,10 +5242,10 @@
         <v>3.63</v>
       </c>
       <c r="J48" t="n">
-        <v>5.123</v>
+        <v>5.227</v>
       </c>
       <c r="K48" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="L48" t="n">
         <v>30</v>
@@ -5290,7 +5309,7 @@
         <v>4.34</v>
       </c>
       <c r="J49" t="n">
-        <v>7.855</v>
+        <v>8.111000000000001</v>
       </c>
       <c r="K49" t="n">
         <v>0.008</v>
@@ -5357,10 +5376,10 @@
         <v>3.24</v>
       </c>
       <c r="J50" t="n">
-        <v>5.727</v>
+        <v>5.591</v>
       </c>
       <c r="K50" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="L50" t="n">
         <v>32</v>
@@ -5424,10 +5443,10 @@
         <v>8.640000000000001</v>
       </c>
       <c r="J51" t="n">
-        <v>14.909</v>
+        <v>15.186</v>
       </c>
       <c r="K51" t="n">
-        <v>0.012</v>
+        <v>0.017</v>
       </c>
       <c r="L51" t="n">
         <v>89</v>
@@ -5491,10 +5510,10 @@
         <v>3.24</v>
       </c>
       <c r="J52" t="n">
-        <v>5.429</v>
+        <v>5.488</v>
       </c>
       <c r="K52" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
       <c r="L52" t="n">
         <v>32</v>
@@ -5566,10 +5585,10 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>4181.678</v>
+        <v>4327.236</v>
       </c>
       <c r="K53" t="n">
-        <v>3.391</v>
+        <v>3.574</v>
       </c>
       <c r="L53" t="n">
         <v>25200</v>
@@ -5649,10 +5668,10 @@
         <v>91.45</v>
       </c>
       <c r="J54" t="n">
-        <v>164.735</v>
+        <v>183.129</v>
       </c>
       <c r="K54" t="n">
-        <v>0.122</v>
+        <v>0.119</v>
       </c>
       <c r="L54" t="n">
         <v>959</v>
@@ -5716,10 +5735,10 @@
         <v>126.66</v>
       </c>
       <c r="J55" t="n">
-        <v>218.743</v>
+        <v>223.727</v>
       </c>
       <c r="K55" t="n">
-        <v>0.182</v>
+        <v>0.18</v>
       </c>
       <c r="L55" t="n">
         <v>1330</v>
@@ -5783,10 +5802,10 @@
         <v>48.44</v>
       </c>
       <c r="J56" t="n">
-        <v>80.90600000000001</v>
+        <v>81.444</v>
       </c>
       <c r="K56" t="n">
-        <v>0.064</v>
+        <v>0.067</v>
       </c>
       <c r="L56" t="n">
         <v>490</v>
@@ -5850,10 +5869,10 @@
         <v>881.71</v>
       </c>
       <c r="J57" t="n">
-        <v>1466.321</v>
+        <v>1486.619</v>
       </c>
       <c r="K57" t="n">
-        <v>1.092</v>
+        <v>1.093</v>
       </c>
       <c r="L57" t="n">
         <v>8831</v>
@@ -5933,7 +5952,7 @@
         <v>11.81</v>
       </c>
       <c r="J58" t="n">
-        <v>17.687</v>
+        <v>18.158</v>
       </c>
       <c r="K58" t="n">
         <v>0.032</v>
@@ -6000,10 +6019,10 @@
         <v>30.63</v>
       </c>
       <c r="J59" t="n">
-        <v>51.18</v>
+        <v>52.957</v>
       </c>
       <c r="K59" t="n">
-        <v>0.055</v>
+        <v>0.056</v>
       </c>
       <c r="L59" t="n">
         <v>298</v>
@@ -6067,10 +6086,10 @@
         <v>1361.3</v>
       </c>
       <c r="J60" t="n">
-        <v>2055.169</v>
+        <v>2090.174</v>
       </c>
       <c r="K60" t="n">
-        <v>1.872</v>
+        <v>1.924</v>
       </c>
       <c r="L60" t="n">
         <v>12456</v>
@@ -6150,10 +6169,10 @@
         <v>69.3</v>
       </c>
       <c r="J61" t="n">
-        <v>119.446</v>
+        <v>121.989</v>
       </c>
       <c r="K61" t="n">
-        <v>0.097</v>
+        <v>0.095</v>
       </c>
       <c r="L61" t="n">
         <v>716</v>
@@ -6217,10 +6236,10 @@
         <v>459.18</v>
       </c>
       <c r="J62" t="n">
-        <v>785.268</v>
+        <v>795.775</v>
       </c>
       <c r="K62" t="n">
-        <v>0.607</v>
+        <v>0.572</v>
       </c>
       <c r="L62" t="n">
         <v>4732</v>
@@ -6228,25 +6247,17 @@
       <c r="M62" t="n">
         <v>460.22</v>
       </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="N62" t="n">
+        <v>58071</v>
+      </c>
+      <c r="O62" t="n">
+        <v>211.5</v>
+      </c>
+      <c r="P62" t="n">
+        <v>2676</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>292.1</v>
       </c>
       <c r="R62" t="n">
         <v>57788.5</v>
@@ -6292,10 +6303,10 @@
         <v>137.14</v>
       </c>
       <c r="J63" t="n">
-        <v>243.568</v>
+        <v>244.973</v>
       </c>
       <c r="K63" t="n">
-        <v>0.182</v>
+        <v>0.185</v>
       </c>
       <c r="L63" t="n">
         <v>1471</v>
@@ -6359,10 +6370,10 @@
         <v>728.2</v>
       </c>
       <c r="J64" t="n">
-        <v>1325.898</v>
+        <v>1226.302</v>
       </c>
       <c r="K64" t="n">
-        <v>0.904</v>
+        <v>0.908</v>
       </c>
       <c r="L64" t="n">
         <v>7349</v>
@@ -6450,10 +6461,10 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>4662.379</v>
+        <v>4784.742</v>
       </c>
       <c r="K65" t="n">
-        <v>3.621</v>
+        <v>3.632</v>
       </c>
       <c r="L65" t="n">
         <v>27842</v>
@@ -6533,10 +6544,10 @@
         <v>1.7</v>
       </c>
       <c r="J66" t="n">
-        <v>3.213</v>
+        <v>3.173</v>
       </c>
       <c r="K66" t="n">
-        <v>0.003</v>
+        <v>0.011</v>
       </c>
       <c r="L66" t="n">
         <v>18</v>
@@ -6600,7 +6611,7 @@
         <v>1.13</v>
       </c>
       <c r="J67" t="n">
-        <v>1.665</v>
+        <v>1.818</v>
       </c>
       <c r="K67" t="n">
         <v>0.002</v>
@@ -6667,10 +6678,10 @@
         <v>46.82</v>
       </c>
       <c r="J68" t="n">
-        <v>82.643</v>
+        <v>83.19199999999999</v>
       </c>
       <c r="K68" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="L68" t="n">
         <v>490</v>
@@ -6734,10 +6745,10 @@
         <v>30.23</v>
       </c>
       <c r="J69" t="n">
-        <v>53.058</v>
+        <v>54.771</v>
       </c>
       <c r="K69" t="n">
-        <v>0.041</v>
+        <v>0.036</v>
       </c>
       <c r="L69" t="n">
         <v>315</v>
@@ -6801,10 +6812,10 @@
         <v>89.05</v>
       </c>
       <c r="J70" t="n">
-        <v>153.371</v>
+        <v>155.516</v>
       </c>
       <c r="K70" t="n">
-        <v>0.116</v>
+        <v>0.11</v>
       </c>
       <c r="L70" t="n">
         <v>933</v>
@@ -6868,7 +6879,7 @@
         <v>1.12</v>
       </c>
       <c r="J71" t="n">
-        <v>1.787</v>
+        <v>1.778</v>
       </c>
       <c r="K71" t="n">
         <v>0.002</v>
@@ -6966,25 +6977,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="R72" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="S72" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="T72" t="n">
+        <v>1</v>
+      </c>
+      <c r="U72" t="n">
+        <v>0.09</v>
       </c>
     </row>
     <row r="73">
@@ -7018,10 +7021,10 @@
         <v>664.5</v>
       </c>
       <c r="J73" t="n">
-        <v>1129.262</v>
+        <v>1166.442</v>
       </c>
       <c r="K73" t="n">
-        <v>0.833</v>
+        <v>0.963</v>
       </c>
       <c r="L73" t="n">
         <v>6771</v>
@@ -7101,10 +7104,10 @@
         <v>1.7</v>
       </c>
       <c r="J74" t="n">
-        <v>3</v>
+        <v>3.159</v>
       </c>
       <c r="K74" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="L74" t="n">
         <v>18</v>
@@ -7168,10 +7171,10 @@
         <v>25.77</v>
       </c>
       <c r="J75" t="n">
-        <v>45.47</v>
+        <v>46.557</v>
       </c>
       <c r="K75" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
       <c r="L75" t="n">
         <v>264</v>
@@ -7235,10 +7238,10 @@
         <v>18.09</v>
       </c>
       <c r="J76" t="n">
-        <v>32.368</v>
+        <v>33.455</v>
       </c>
       <c r="K76" t="n">
-        <v>0.027</v>
+        <v>0.035</v>
       </c>
       <c r="L76" t="n">
         <v>191</v>
@@ -7302,10 +7305,10 @@
         <v>103.08</v>
       </c>
       <c r="J77" t="n">
-        <v>184.236</v>
+        <v>184.543</v>
       </c>
       <c r="K77" t="n">
-        <v>0.118</v>
+        <v>0.116</v>
       </c>
       <c r="L77" t="n">
         <v>1080</v>
@@ -7369,10 +7372,10 @@
         <v>493.87</v>
       </c>
       <c r="J78" t="n">
-        <v>894.045</v>
+        <v>910.578</v>
       </c>
       <c r="K78" t="n">
-        <v>0.541</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L78" t="n">
         <v>5180</v>
@@ -7380,25 +7383,17 @@
       <c r="M78" t="n">
         <v>489.77</v>
       </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q78" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="N78" t="n">
+        <v>46298.7</v>
+      </c>
+      <c r="O78" t="n">
+        <v>209.6</v>
+      </c>
+      <c r="P78" t="n">
+        <v>2972</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>314.16</v>
       </c>
       <c r="R78" t="n">
         <v>47868.3</v>
@@ -7444,10 +7439,10 @@
         <v>1786.36</v>
       </c>
       <c r="J79" t="n">
-        <v>3160.001</v>
+        <v>3239.493</v>
       </c>
       <c r="K79" t="n">
-        <v>2.241</v>
+        <v>2.228</v>
       </c>
       <c r="L79" t="n">
         <v>18622</v>
@@ -7535,10 +7530,10 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>9090.190000000001</v>
+        <v>9240.5</v>
       </c>
       <c r="K80" t="n">
-        <v>6.585</v>
+        <v>7.352</v>
       </c>
       <c r="L80" t="n">
         <v>53727</v>
@@ -7626,10 +7621,10 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>27325.809</v>
+        <v>27680.628</v>
       </c>
       <c r="K81" t="n">
-        <v>21.765</v>
+        <v>22.36</v>
       </c>
       <c r="L81" t="n">
         <v>161192</v>
@@ -7709,10 +7704,10 @@
         <v>796.26</v>
       </c>
       <c r="J82" t="n">
-        <v>1351.206</v>
+        <v>1360.76</v>
       </c>
       <c r="K82" t="n">
-        <v>0.982</v>
+        <v>1.044</v>
       </c>
       <c r="L82" t="n">
         <v>8147</v>
@@ -7792,10 +7787,10 @@
         <v>5.55</v>
       </c>
       <c r="J83" t="n">
-        <v>9.989000000000001</v>
+        <v>10.126</v>
       </c>
       <c r="K83" t="n">
-        <v>0.031</v>
+        <v>0.027</v>
       </c>
       <c r="L83" t="n">
         <v>36</v>
@@ -7859,10 +7854,10 @@
         <v>7.79</v>
       </c>
       <c r="J84" t="n">
-        <v>14.208</v>
+        <v>13.623</v>
       </c>
       <c r="K84" t="n">
-        <v>0.066</v>
+        <v>0.042</v>
       </c>
       <c r="L84" t="n">
         <v>49</v>
@@ -7926,10 +7921,10 @@
         <v>7.8</v>
       </c>
       <c r="J85" t="n">
-        <v>15.751</v>
+        <v>15.857</v>
       </c>
       <c r="K85" t="n">
-        <v>0.062</v>
+        <v>0.074</v>
       </c>
       <c r="L85" t="n">
         <v>61</v>
@@ -7993,10 +7988,10 @@
         <v>1700.66</v>
       </c>
       <c r="J86" t="n">
-        <v>2922.598</v>
+        <v>2948.696</v>
       </c>
       <c r="K86" t="n">
-        <v>2.05</v>
+        <v>2.111</v>
       </c>
       <c r="L86" t="n">
         <v>17374</v>
@@ -8076,10 +8071,10 @@
         <v>46.73</v>
       </c>
       <c r="J87" t="n">
-        <v>79.04300000000001</v>
+        <v>79.866</v>
       </c>
       <c r="K87" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.061</v>
       </c>
       <c r="L87" t="n">
         <v>472</v>
@@ -8143,10 +8138,10 @@
         <v>1998.55</v>
       </c>
       <c r="J88" t="n">
-        <v>3413.629</v>
+        <v>3449.893</v>
       </c>
       <c r="K88" t="n">
-        <v>2.677</v>
+        <v>2.426</v>
       </c>
       <c r="L88" t="n">
         <v>20132</v>
@@ -8226,10 +8221,10 @@
         <v>4.25</v>
       </c>
       <c r="J89" t="n">
-        <v>7.555</v>
+        <v>7.797</v>
       </c>
       <c r="K89" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="L89" t="n">
         <v>46</v>
@@ -8293,10 +8288,10 @@
         <v>24.05</v>
       </c>
       <c r="J90" t="n">
-        <v>38.626</v>
+        <v>38.911</v>
       </c>
       <c r="K90" t="n">
-        <v>0.028</v>
+        <v>0.03</v>
       </c>
       <c r="L90" t="n">
         <v>225</v>
@@ -8360,10 +8355,10 @@
         <v>12.57</v>
       </c>
       <c r="J91" t="n">
-        <v>19.2</v>
+        <v>18.991</v>
       </c>
       <c r="K91" t="n">
-        <v>0.022</v>
+        <v>0.024</v>
       </c>
       <c r="L91" t="n">
         <v>117</v>
@@ -8427,10 +8422,10 @@
         <v>361.88</v>
       </c>
       <c r="J92" t="n">
-        <v>615.397</v>
+        <v>624.854</v>
       </c>
       <c r="K92" t="n">
-        <v>0.435</v>
+        <v>0.452</v>
       </c>
       <c r="L92" t="n">
         <v>3709</v>
@@ -8438,25 +8433,17 @@
       <c r="M92" t="n">
         <v>365.35</v>
       </c>
-      <c r="N92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="N92" t="n">
+        <v>52044.5</v>
+      </c>
+      <c r="O92" t="n">
+        <v>173.3</v>
+      </c>
+      <c r="P92" t="n">
+        <v>2083</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>236.25</v>
       </c>
       <c r="R92" t="n">
         <v>48998.7</v>
@@ -8502,10 +8489,10 @@
         <v>1439.87</v>
       </c>
       <c r="J93" t="n">
-        <v>2415.28</v>
+        <v>2407.826</v>
       </c>
       <c r="K93" t="n">
-        <v>1.803</v>
+        <v>1.732</v>
       </c>
       <c r="L93" t="n">
         <v>14460</v>
@@ -8585,10 +8572,10 @@
         <v>18.99</v>
       </c>
       <c r="J94" t="n">
-        <v>33.996</v>
+        <v>33.36</v>
       </c>
       <c r="K94" t="n">
-        <v>0.029</v>
+        <v>0.026</v>
       </c>
       <c r="L94" t="n">
         <v>196</v>
@@ -8652,10 +8639,10 @@
         <v>13.41</v>
       </c>
       <c r="J95" t="n">
-        <v>25.174</v>
+        <v>24.847</v>
       </c>
       <c r="K95" t="n">
-        <v>0.023</v>
+        <v>0.02</v>
       </c>
       <c r="L95" t="n">
         <v>137</v>
@@ -8719,10 +8706,10 @@
         <v>41.23</v>
       </c>
       <c r="J96" t="n">
-        <v>71.71299999999999</v>
+        <v>72.654</v>
       </c>
       <c r="K96" t="n">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="L96" t="n">
         <v>419</v>
@@ -8786,10 +8773,10 @@
         <v>3.01</v>
       </c>
       <c r="J97" t="n">
-        <v>4.292</v>
+        <v>4.127</v>
       </c>
       <c r="K97" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
       <c r="L97" t="n">
         <v>24</v>
@@ -8853,10 +8840,10 @@
         <v>4.73</v>
       </c>
       <c r="J98" t="n">
-        <v>8.281000000000001</v>
+        <v>8.204000000000001</v>
       </c>
       <c r="K98" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="L98" t="n">
         <v>50</v>
@@ -8920,10 +8907,10 @@
         <v>3.1</v>
       </c>
       <c r="J99" t="n">
-        <v>5.5</v>
+        <v>5.525</v>
       </c>
       <c r="K99" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="L99" t="n">
         <v>32</v>
@@ -8987,7 +8974,7 @@
         <v>34.23</v>
       </c>
       <c r="J100" t="n">
-        <v>59.593</v>
+        <v>60.18</v>
       </c>
       <c r="K100" t="n">
         <v>0.04</v>
@@ -9054,10 +9041,10 @@
         <v>26.56</v>
       </c>
       <c r="J101" t="n">
-        <v>46.516</v>
+        <v>48.088</v>
       </c>
       <c r="K101" t="n">
-        <v>0.036</v>
+        <v>0.034</v>
       </c>
       <c r="L101" t="n">
         <v>273</v>
@@ -9121,10 +9108,10 @@
         <v>22.33</v>
       </c>
       <c r="J102" t="n">
-        <v>39.88</v>
+        <v>40.645</v>
       </c>
       <c r="K102" t="n">
-        <v>0.031</v>
+        <v>0.032</v>
       </c>
       <c r="L102" t="n">
         <v>236</v>
@@ -9188,10 +9175,10 @@
         <v>11.74</v>
       </c>
       <c r="J103" t="n">
-        <v>20.649</v>
+        <v>20.712</v>
       </c>
       <c r="K103" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="L103" t="n">
         <v>116</v>
@@ -9255,10 +9242,10 @@
         <v>10.77</v>
       </c>
       <c r="J104" t="n">
-        <v>18.951</v>
+        <v>19.201</v>
       </c>
       <c r="K104" t="n">
-        <v>0.016</v>
+        <v>0.015</v>
       </c>
       <c r="L104" t="n">
         <v>113</v>
@@ -9322,7 +9309,7 @@
         <v>6.55</v>
       </c>
       <c r="J105" t="n">
-        <v>10.544</v>
+        <v>10.519</v>
       </c>
       <c r="K105" t="n">
         <v>0.011</v>
@@ -9389,10 +9376,10 @@
         <v>7.36</v>
       </c>
       <c r="J106" t="n">
-        <v>10.479</v>
+        <v>10.314</v>
       </c>
       <c r="K106" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="L106" t="n">
         <v>61</v>
@@ -9464,10 +9451,10 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>16960.865</v>
+        <v>17054.889</v>
       </c>
       <c r="K107" t="n">
-        <v>12.655</v>
+        <v>13.662</v>
       </c>
       <c r="L107" t="n">
         <v>100335</v>
@@ -9555,10 +9542,10 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>24575.506</v>
+        <v>24723.016</v>
       </c>
       <c r="K108" t="n">
-        <v>21.582</v>
+        <v>21.632</v>
       </c>
       <c r="L108" t="n">
         <v>146003</v>
@@ -9638,10 +9625,10 @@
         <v>126.66</v>
       </c>
       <c r="J109" t="n">
-        <v>220.052</v>
+        <v>221.939</v>
       </c>
       <c r="K109" t="n">
-        <v>0.195</v>
+        <v>0.181</v>
       </c>
       <c r="L109" t="n">
         <v>1330</v>
@@ -9705,7 +9692,7 @@
         <v>2.21</v>
       </c>
       <c r="J110" t="n">
-        <v>5.997</v>
+        <v>6.157</v>
       </c>
       <c r="K110" t="n">
         <v>0.005</v>
@@ -9772,10 +9759,10 @@
         <v>2.18</v>
       </c>
       <c r="J111" t="n">
-        <v>6.349</v>
+        <v>6.7</v>
       </c>
       <c r="K111" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="L111" t="n">
         <v>18</v>
@@ -10021,10 +10008,10 @@
         <v>244.53</v>
       </c>
       <c r="J114" t="n">
-        <v>416.449</v>
+        <v>423.015</v>
       </c>
       <c r="K114" t="n">
-        <v>0.324</v>
+        <v>0.316</v>
       </c>
       <c r="L114" t="n">
         <v>2498</v>
@@ -10088,10 +10075,10 @@
         <v>2.3</v>
       </c>
       <c r="J115" t="n">
-        <v>4.01</v>
+        <v>4.318</v>
       </c>
       <c r="K115" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="L115" t="n">
         <v>24</v>
@@ -10155,10 +10142,10 @@
         <v>2.3</v>
       </c>
       <c r="J116" t="n">
-        <v>4.273</v>
+        <v>4.182</v>
       </c>
       <c r="K116" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="L116" t="n">
         <v>24</v>
@@ -10222,10 +10209,10 @@
         <v>6.41</v>
       </c>
       <c r="J117" t="n">
-        <v>11.722</v>
+        <v>12.41</v>
       </c>
       <c r="K117" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="L117" t="n">
         <v>68</v>
@@ -10289,10 +10276,10 @@
         <v>74.3</v>
       </c>
       <c r="J118" t="n">
-        <v>133.857</v>
+        <v>135.936</v>
       </c>
       <c r="K118" t="n">
-        <v>0.097</v>
+        <v>0.099</v>
       </c>
       <c r="L118" t="n">
         <v>784</v>
@@ -10356,10 +10343,10 @@
         <v>34.93</v>
       </c>
       <c r="J119" t="n">
-        <v>59.657</v>
+        <v>61.333</v>
       </c>
       <c r="K119" t="n">
-        <v>0.048</v>
+        <v>0.051</v>
       </c>
       <c r="L119" t="n">
         <v>357</v>
@@ -10423,10 +10410,10 @@
         <v>42.34</v>
       </c>
       <c r="J120" t="n">
-        <v>76.8</v>
+        <v>78.575</v>
       </c>
       <c r="K120" t="n">
-        <v>0.06</v>
+        <v>0.063</v>
       </c>
       <c r="L120" t="n">
         <v>445</v>
@@ -10490,10 +10477,10 @@
         <v>21.87</v>
       </c>
       <c r="J121" t="n">
-        <v>39.731</v>
+        <v>40.471</v>
       </c>
       <c r="K121" t="n">
-        <v>0.034</v>
+        <v>0.031</v>
       </c>
       <c r="L121" t="n">
         <v>228</v>
@@ -10557,10 +10544,10 @@
         <v>10.03</v>
       </c>
       <c r="J122" t="n">
-        <v>14.941</v>
+        <v>15.177</v>
       </c>
       <c r="K122" t="n">
-        <v>0.016</v>
+        <v>0.018</v>
       </c>
       <c r="L122" t="n">
         <v>88</v>
@@ -10624,10 +10611,10 @@
         <v>94.54000000000001</v>
       </c>
       <c r="J123" t="n">
-        <v>170.551</v>
+        <v>176.885</v>
       </c>
       <c r="K123" t="n">
-        <v>0.122</v>
+        <v>0.119</v>
       </c>
       <c r="L123" t="n">
         <v>1012</v>
@@ -10691,10 +10678,10 @@
         <v>19.55</v>
       </c>
       <c r="J124" t="n">
-        <v>32.421</v>
+        <v>32.941</v>
       </c>
       <c r="K124" t="n">
-        <v>0.04</v>
+        <v>0.038</v>
       </c>
       <c r="L124" t="n">
         <v>203</v>
@@ -10758,10 +10745,10 @@
         <v>15.67</v>
       </c>
       <c r="J125" t="n">
-        <v>24.687</v>
+        <v>24.495</v>
       </c>
       <c r="K125" t="n">
-        <v>0.027</v>
+        <v>0.033</v>
       </c>
       <c r="L125" t="n">
         <v>148</v>
@@ -10825,10 +10812,10 @@
         <v>391.16</v>
       </c>
       <c r="J126" t="n">
-        <v>678.495</v>
+        <v>692.741</v>
       </c>
       <c r="K126" t="n">
-        <v>0.49</v>
+        <v>0.489</v>
       </c>
       <c r="L126" t="n">
         <v>4048</v>
@@ -10836,25 +10823,17 @@
       <c r="M126" t="n">
         <v>390.21</v>
       </c>
-      <c r="N126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="N126" t="n">
+        <v>45926.9</v>
+      </c>
+      <c r="O126" t="n">
+        <v>182.6</v>
+      </c>
+      <c r="P126" t="n">
+        <v>2355</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>260.89</v>
       </c>
       <c r="R126" t="n">
         <v>45187.2</v>
@@ -10900,10 +10879,10 @@
         <v>27.98</v>
       </c>
       <c r="J127" t="n">
-        <v>30.932</v>
+        <v>31.727</v>
       </c>
       <c r="K127" t="n">
-        <v>0.046</v>
+        <v>0.049</v>
       </c>
       <c r="L127" t="n">
         <v>183</v>
@@ -10967,10 +10946,10 @@
         <v>1012.04</v>
       </c>
       <c r="J128" t="n">
-        <v>1725.722</v>
+        <v>1742.598</v>
       </c>
       <c r="K128" t="n">
-        <v>1.384</v>
+        <v>2.187</v>
       </c>
       <c r="L128" t="n">
         <v>10305</v>
@@ -11050,10 +11029,10 @@
         <v>1277.49</v>
       </c>
       <c r="J129" t="n">
-        <v>2102.246</v>
+        <v>2139.987</v>
       </c>
       <c r="K129" t="n">
-        <v>1.632</v>
+        <v>1.686</v>
       </c>
       <c r="L129" t="n">
         <v>12565</v>
@@ -11141,10 +11120,10 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>4659.138</v>
+        <v>4770.623</v>
       </c>
       <c r="K130" t="n">
-        <v>3.832</v>
+        <v>4.205</v>
       </c>
       <c r="L130" t="n">
         <v>27939</v>
@@ -11224,10 +11203,10 @@
         <v>57.6</v>
       </c>
       <c r="J131" t="n">
-        <v>101.953</v>
+        <v>104.211</v>
       </c>
       <c r="K131" t="n">
-        <v>0.066</v>
+        <v>0.064</v>
       </c>
       <c r="L131" t="n">
         <v>600</v>
@@ -11291,10 +11270,10 @@
         <v>57.96</v>
       </c>
       <c r="J132" t="n">
-        <v>102.859</v>
+        <v>105.202</v>
       </c>
       <c r="K132" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L132" t="n">
         <v>604</v>
@@ -11358,10 +11337,10 @@
         <v>737.08</v>
       </c>
       <c r="J133" t="n">
-        <v>1288.699</v>
+        <v>1295.713</v>
       </c>
       <c r="K133" t="n">
-        <v>0.905</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="L133" t="n">
         <v>7746</v>
@@ -11441,10 +11420,10 @@
         <v>225.86</v>
       </c>
       <c r="J134" t="n">
-        <v>390.825</v>
+        <v>395.307</v>
       </c>
       <c r="K134" t="n">
-        <v>0.285</v>
+        <v>0.29</v>
       </c>
       <c r="L134" t="n">
         <v>2322</v>
@@ -11508,10 +11487,10 @@
         <v>144.95</v>
       </c>
       <c r="J135" t="n">
-        <v>248.301</v>
+        <v>255.189</v>
       </c>
       <c r="K135" t="n">
-        <v>0.2</v>
+        <v>0.209</v>
       </c>
       <c r="L135" t="n">
         <v>1487</v>
@@ -11575,10 +11554,10 @@
         <v>533.46</v>
       </c>
       <c r="J136" t="n">
-        <v>886.148</v>
+        <v>900.249</v>
       </c>
       <c r="K136" t="n">
-        <v>0.744</v>
+        <v>0.738</v>
       </c>
       <c r="L136" t="n">
         <v>5359</v>
@@ -11666,10 +11645,10 @@
         </is>
       </c>
       <c r="J137" t="n">
-        <v>8351.005999999999</v>
+        <v>8437.407999999999</v>
       </c>
       <c r="K137" t="n">
-        <v>6.082</v>
+        <v>6.252</v>
       </c>
       <c r="L137" t="n">
         <v>49505</v>
@@ -11749,10 +11728,10 @@
         <v>289.33</v>
       </c>
       <c r="J138" t="n">
-        <v>519.639</v>
+        <v>529.901</v>
       </c>
       <c r="K138" t="n">
-        <v>0.354</v>
+        <v>0.331</v>
       </c>
       <c r="L138" t="n">
         <v>3059</v>
@@ -11816,10 +11795,10 @@
         <v>21</v>
       </c>
       <c r="J139" t="n">
-        <v>34.357</v>
+        <v>34.864</v>
       </c>
       <c r="K139" t="n">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="L139" t="n">
         <v>207</v>
@@ -11883,10 +11862,10 @@
         <v>23.1</v>
       </c>
       <c r="J140" t="n">
-        <v>33.244</v>
+        <v>33.331</v>
       </c>
       <c r="K140" t="n">
-        <v>0.044</v>
+        <v>0.042</v>
       </c>
       <c r="L140" t="n">
         <v>208</v>
@@ -11950,10 +11929,10 @@
         <v>1592.96</v>
       </c>
       <c r="J141" t="n">
-        <v>2817.208</v>
+        <v>2869.918</v>
       </c>
       <c r="K141" t="n">
-        <v>1.83</v>
+        <v>1.829</v>
       </c>
       <c r="L141" t="n">
         <v>16621</v>
@@ -12041,10 +12020,10 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>4602.981</v>
+        <v>4569.241</v>
       </c>
       <c r="K142" t="n">
-        <v>3.042</v>
+        <v>3.22</v>
       </c>
       <c r="L142" t="n">
         <v>26800</v>
@@ -12124,10 +12103,10 @@
         <v>16.28</v>
       </c>
       <c r="J143" t="n">
-        <v>20.089</v>
+        <v>20.552</v>
       </c>
       <c r="K143" t="n">
-        <v>0.024</v>
+        <v>0.029</v>
       </c>
       <c r="L143" t="n">
         <v>121</v>
@@ -12199,10 +12178,10 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>25005.324</v>
+        <v>25297.491</v>
       </c>
       <c r="K144" t="n">
-        <v>16.903</v>
+        <v>21.061</v>
       </c>
       <c r="L144" t="n">
         <v>140783</v>
@@ -12290,10 +12269,10 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>7890.297</v>
+        <v>7958.599</v>
       </c>
       <c r="K145" t="n">
-        <v>5.733</v>
+        <v>5.876</v>
       </c>
       <c r="L145" t="n">
         <v>46451</v>
@@ -12381,10 +12360,10 @@
         </is>
       </c>
       <c r="J146" t="n">
-        <v>11048.168</v>
+        <v>11126.794</v>
       </c>
       <c r="K146" t="n">
-        <v>7.017</v>
+        <v>6.368</v>
       </c>
       <c r="L146" t="n">
         <v>62186</v>
@@ -12464,10 +12443,10 @@
         <v>1673.66</v>
       </c>
       <c r="J147" t="n">
-        <v>2951.269</v>
+        <v>2941.937</v>
       </c>
       <c r="K147" t="n">
-        <v>2.28</v>
+        <v>2.105</v>
       </c>
       <c r="L147" t="n">
         <v>17253</v>
@@ -12555,10 +12534,10 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>57125.052</v>
+        <v>57382.181</v>
       </c>
       <c r="K148" t="n">
-        <v>41.594</v>
+        <v>39.04</v>
       </c>
       <c r="L148" t="n">
         <v>323821</v>
@@ -12646,10 +12625,10 @@
         </is>
       </c>
       <c r="J149" t="n">
-        <v>17715.535</v>
+        <v>17832.866</v>
       </c>
       <c r="K149" t="n">
-        <v>13.338</v>
+        <v>13.689</v>
       </c>
       <c r="L149" t="n">
         <v>105486</v>
@@ -12737,10 +12716,10 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>64988.813</v>
+        <v>65372.193</v>
       </c>
       <c r="K150" t="n">
-        <v>52.908</v>
+        <v>50.369</v>
       </c>
       <c r="L150" t="n">
         <v>375160</v>
@@ -12828,10 +12807,10 @@
         </is>
       </c>
       <c r="J151" t="n">
-        <v>22049.624</v>
+        <v>23104.825</v>
       </c>
       <c r="K151" t="n">
-        <v>14.18</v>
+        <v>13.792</v>
       </c>
       <c r="L151" t="n">
         <v>125533</v>
@@ -12919,10 +12898,10 @@
         </is>
       </c>
       <c r="J152" t="n">
-        <v>6962.157</v>
+        <v>7090.603</v>
       </c>
       <c r="K152" t="n">
-        <v>5.099</v>
+        <v>5.333</v>
       </c>
       <c r="L152" t="n">
         <v>41254</v>
@@ -13010,10 +12989,10 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>22913.807</v>
+        <v>23038.568</v>
       </c>
       <c r="K153" t="n">
-        <v>16.887</v>
+        <v>16.258</v>
       </c>
       <c r="L153" t="n">
         <v>130961</v>
@@ -13093,10 +13072,10 @@
         <v>68.75</v>
       </c>
       <c r="J154" t="n">
-        <v>122.585</v>
+        <v>125.332</v>
       </c>
       <c r="K154" t="n">
-        <v>0.103</v>
+        <v>0.107</v>
       </c>
       <c r="L154" t="n">
         <v>728</v>
@@ -13160,10 +13139,10 @@
         <v>1.13</v>
       </c>
       <c r="J155" t="n">
-        <v>1.686</v>
+        <v>1.692</v>
       </c>
       <c r="K155" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="L155" t="n">
         <v>10</v>
@@ -13227,10 +13206,10 @@
         <v>226.66</v>
       </c>
       <c r="J156" t="n">
-        <v>395.411</v>
+        <v>391.399</v>
       </c>
       <c r="K156" t="n">
-        <v>0.301</v>
+        <v>0.312</v>
       </c>
       <c r="L156" t="n">
         <v>2314</v>
@@ -13273,13 +13252,13 @@
         <v>1830495.2</v>
       </c>
       <c r="C158" t="n">
-        <v>385168.3</v>
+        <v>389366.5</v>
       </c>
       <c r="D158" t="n">
-        <v>405991.3</v>
+        <v>608332.4</v>
       </c>
       <c r="E158" t="n">
-        <v>600396.3</v>
+        <v>600430.2</v>
       </c>
     </row>
     <row r="159">
@@ -13292,13 +13271,13 @@
         <v>11124.7</v>
       </c>
       <c r="C159" t="n">
-        <v>290.4</v>
+        <v>292.3</v>
       </c>
       <c r="D159" t="n">
-        <v>1825.3</v>
+        <v>2602.3</v>
       </c>
       <c r="E159" t="n">
-        <v>2639.1</v>
+        <v>2639.2</v>
       </c>
     </row>
     <row r="160">
@@ -13314,10 +13293,10 @@
         <v>2237491</v>
       </c>
       <c r="D160" t="n">
-        <v>22764</v>
+        <v>32850</v>
       </c>
       <c r="E160" t="n">
-        <v>32420</v>
+        <v>32421</v>
       </c>
     </row>
     <row r="161">
@@ -13333,48 +13312,67 @@
         <v>215730.3</v>
       </c>
       <c r="D161" t="n">
-        <v>2470.4</v>
+        <v>3573.8</v>
       </c>
       <c r="E161" t="n">
-        <v>3521.7</v>
+        <v>3521.8</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>geomean Steps/ZAC</t>
+          <t>平均保真度(四法齐全 N=117)</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>1</v>
+        <v>0.4288</v>
       </c>
       <c r="C162" t="n">
-        <v>0.97</v>
+        <v>0.4282</v>
       </c>
       <c r="D162" t="n">
-        <v>0.595</v>
+        <v>0.4744</v>
       </c>
       <c r="E162" t="n">
-        <v>0.59</v>
+        <v>0.4747</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>geomean Rearr/ZAC</t>
+          <t>geomean Steps/ZAC</t>
         </is>
       </c>
       <c r="B163" t="n">
         <v>1</v>
       </c>
       <c r="C163" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0.594</v>
+      </c>
+      <c r="E163" t="n">
+        <v>0.589</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>geomean Rearr/ZAC</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>1</v>
+      </c>
+      <c r="C164" t="n">
         <v>0.973</v>
       </c>
-      <c r="D163" t="n">
+      <c r="D164" t="n">
         <v>0.652</v>
       </c>
-      <c r="E163" t="n">
-        <v>0.647</v>
+      <c r="E164" t="n">
+        <v>0.645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>